<commit_message>
Add helper to log a variable description.
</commit_message>
<xml_diff>
--- a/VVariables.xlsx
+++ b/VVariables.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3B1646-63C3-48B5-B64F-9D9120F75840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5DE43A-CDB7-4B21-BE3C-D775B3DBFF15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F3308010-532B-49A6-9B56-20C10732166F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F3308010-532B-49A6-9B56-20C10732166F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1 (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
   <si>
     <t>Fixed at 'F'</t>
   </si>
@@ -54,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color theme="1"/>
@@ -70,6 +71,11 @@
     <font>
       <sz val="9"/>
       <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -98,7 +104,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -141,13 +147,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -173,22 +188,37 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -570,7 +600,7 @@
       <c r="A3" s="1">
         <v>0</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="11">
         <v>0</v>
       </c>
       <c r="D3" s="2"/>
@@ -589,7 +619,7 @@
       <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="11">
         <v>0</v>
       </c>
       <c r="D4" s="2"/>
@@ -608,7 +638,7 @@
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="11">
         <v>0</v>
       </c>
       <c r="D5" s="2"/>
@@ -627,7 +657,7 @@
       <c r="A6" s="1">
         <v>3</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="11">
         <v>0</v>
       </c>
       <c r="D6" s="2"/>
@@ -646,7 +676,7 @@
       <c r="A7" s="1">
         <v>4</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="12">
         <v>1</v>
       </c>
       <c r="D7" s="5"/>
@@ -665,7 +695,7 @@
       <c r="A8" s="1">
         <v>5</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="11">
         <v>0</v>
       </c>
       <c r="D8" s="5"/>
@@ -680,23 +710,23 @@
         <v>0</v>
       </c>
       <c r="T8" s="8"/>
-      <c r="U8" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
-      <c r="AA8" s="9"/>
-      <c r="AB8" s="9"/>
-      <c r="AC8" s="9"/>
+      <c r="U8" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14"/>
+      <c r="X8" s="14"/>
+      <c r="Y8" s="14"/>
+      <c r="Z8" s="14"/>
+      <c r="AA8" s="14"/>
+      <c r="AB8" s="14"/>
+      <c r="AC8" s="14"/>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>6</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="12">
         <v>1</v>
       </c>
       <c r="D9" s="5"/>
@@ -710,24 +740,24 @@
       <c r="L9" s="6">
         <v>0</v>
       </c>
-      <c r="T9" s="10"/>
-      <c r="U9" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="9"/>
-      <c r="Z9" s="9"/>
-      <c r="AA9" s="9"/>
-      <c r="AB9" s="9"/>
-      <c r="AC9" s="9"/>
+      <c r="T9" s="9"/>
+      <c r="U9" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="V9" s="14"/>
+      <c r="W9" s="14"/>
+      <c r="X9" s="14"/>
+      <c r="Y9" s="14"/>
+      <c r="Z9" s="14"/>
+      <c r="AA9" s="14"/>
+      <c r="AB9" s="14"/>
+      <c r="AC9" s="14"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>7</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="11">
         <v>0</v>
       </c>
       <c r="D10" s="5"/>
@@ -741,24 +771,24 @@
       <c r="L10" s="6">
         <v>0</v>
       </c>
-      <c r="T10" s="11"/>
-      <c r="U10" s="12" t="s">
+      <c r="T10" s="10"/>
+      <c r="U10" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="V10" s="12"/>
-      <c r="W10" s="12"/>
-      <c r="X10" s="12"/>
-      <c r="Y10" s="12"/>
-      <c r="Z10" s="12"/>
-      <c r="AA10" s="12"/>
-      <c r="AB10" s="12"/>
-      <c r="AC10" s="12"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13"/>
+      <c r="X10" s="13"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="13"/>
+      <c r="AB10" s="13"/>
+      <c r="AC10" s="13"/>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>8</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="12">
         <v>1</v>
       </c>
       <c r="D11" s="5"/>
@@ -777,7 +807,7 @@
       <c r="A12" s="1">
         <v>9</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="11">
         <v>0</v>
       </c>
       <c r="D12" s="5"/>
@@ -796,7 +826,7 @@
       <c r="A13" s="1">
         <v>10</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="12">
         <v>1</v>
       </c>
       <c r="D13" s="5"/>
@@ -815,7 +845,7 @@
       <c r="A14" s="1">
         <v>11</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="11">
         <v>0</v>
       </c>
       <c r="D14" s="5"/>
@@ -834,7 +864,7 @@
       <c r="A15" s="1">
         <v>12</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="11">
         <v>0</v>
       </c>
       <c r="D15" s="5"/>
@@ -853,7 +883,7 @@
       <c r="A16" s="1">
         <v>13</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="12">
         <v>1</v>
       </c>
       <c r="D16" s="4"/>
@@ -872,7 +902,7 @@
       <c r="A17" s="1">
         <v>14</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="12">
         <v>1</v>
       </c>
       <c r="D17" s="4"/>
@@ -891,7 +921,7 @@
       <c r="A18" s="1">
         <v>15</v>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="12">
         <v>1</v>
       </c>
       <c r="D18" s="4"/>
@@ -914,4 +944,213 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC414D10-48D6-42D1-884C-44BE33044C76}">
+  <dimension ref="A1:Z11"/>
+  <sheetFormatPr defaultColWidth="2.83203125" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="2.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="C1" s="1">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1">
+        <v>5</v>
+      </c>
+      <c r="I1" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>0</v>
+      </c>
+      <c r="C3" s="11">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="11">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="12">
+        <v>1</v>
+      </c>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="C6" s="12">
+        <v>1</v>
+      </c>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>4</v>
+      </c>
+      <c r="C7" s="12">
+        <v>1</v>
+      </c>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>5</v>
+      </c>
+      <c r="C8" s="12">
+        <v>1</v>
+      </c>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="S8" s="14"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14"/>
+      <c r="X8" s="14"/>
+      <c r="Y8" s="14"/>
+      <c r="Z8" s="14"/>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>6</v>
+      </c>
+      <c r="C9" s="11">
+        <v>0</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="S9" s="14"/>
+      <c r="T9" s="14"/>
+      <c r="U9" s="14"/>
+      <c r="V9" s="14"/>
+      <c r="W9" s="14"/>
+      <c r="X9" s="14"/>
+      <c r="Y9" s="14"/>
+      <c r="Z9" s="14"/>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>7</v>
+      </c>
+      <c r="C10" s="12">
+        <v>1</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13"/>
+      <c r="X10" s="13"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="I11" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="R8:Z8"/>
+    <mergeCell ref="R9:Z9"/>
+    <mergeCell ref="R10:Z10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>